<commit_message>
LIR Anti Detection & Spawn File consolidation
</commit_message>
<xml_diff>
--- a/_OUTPUT--Recruiting_Coord.xlsx
+++ b/_OUTPUT--Recruiting_Coord.xlsx
@@ -71,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -93,6 +93,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -459,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN102"/>
+  <dimension ref="A1:AN109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20.29" customWidth="1" min="1" max="1"/>
@@ -5955,7 +5958,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n"/>
-      <c r="C33" s="6" t="n"/>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/shubham-patel-sap356427</t>
+        </is>
+      </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/talent/profile/AEMAADV7-rMBq5lTm7XaNLk68qrDTxeA7PVficc</t>
@@ -6977,7 +6984,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n"/>
-      <c r="C39" s="6" t="n"/>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/piyush-malviya-7a6382375</t>
+        </is>
+      </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/talent/profile/AEMAAFzIDe4BPucGq8TqheaFYhgboGOh8AJNlUw</t>
@@ -7147,7 +7158,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n"/>
-      <c r="C40" s="6" t="n"/>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/simran-kumari-a29075200</t>
+        </is>
+      </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/talent/profile/AEMAADNEXoEBP8EfpTStSd8WZo0-a0Nc9XGC8wk</t>
@@ -16177,29 +16192,43 @@
       <c r="Z94" s="7" t="n"/>
       <c r="AA94" s="7" t="n"/>
       <c r="AB94" s="7" t="n"/>
-      <c r="AC94" s="7" t="n"/>
-      <c r="AD94" s="7" t="n"/>
-      <c r="AE94" s="7" t="n"/>
-      <c r="AF94" s="7" t="inlineStr">
-        <is>
-          <t>52.8</t>
-        </is>
-      </c>
-      <c r="AG94" s="7" t="n"/>
+      <c r="AC94" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD94" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE94" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF94" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG94" s="7" t="n">
+        <v>52.8</v>
+      </c>
       <c r="AH94" s="7" t="inlineStr">
         <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="AI94" s="7" t="inlineStr">
+        <is>
           <t>F</t>
         </is>
       </c>
-      <c r="AI94" s="7" t="inlineStr">
+      <c r="AJ94" s="7" t="inlineStr">
         <is>
           <t>Hard No</t>
         </is>
       </c>
-      <c r="AJ94" s="7" t="n"/>
       <c r="AK94" s="7" t="n"/>
       <c r="AL94" s="3" t="n"/>
-      <c r="AM94" s="3" t="n"/>
+      <c r="AM94" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
       <c r="AN94" s="3" t="n"/>
     </row>
     <row r="95">
@@ -17585,6 +17614,907 @@
       </c>
       <c r="AN102" s="3" t="n"/>
     </row>
+    <row r="103">
+      <c r="A103" s="8" t="inlineStr">
+        <is>
+          <t>Paras Shah</t>
+        </is>
+      </c>
+      <c r="B103" s="8" t="inlineStr"/>
+      <c r="C103" s="8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/parashah</t>
+        </is>
+      </c>
+      <c r="D103" s="8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/talent/profile/AEMAAB_w53kBJjUA4mGrVR4OZYVK_EGxxZehRIA</t>
+        </is>
+      </c>
+      <c r="E103" s="8" t="inlineStr">
+        <is>
+          <t>Talent Scout Specialist</t>
+        </is>
+      </c>
+      <c r="F103" s="8" t="inlineStr">
+        <is>
+          <t>Accenture</t>
+        </is>
+      </c>
+      <c r="G103" s="8" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat, India</t>
+        </is>
+      </c>
+      <c r="H103" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I103" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J103" s="8" t="inlineStr"/>
+      <c r="K103" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L103" s="8" t="inlineStr">
+        <is>
+          <t>HR generalist/Talent Scout role; recruiting duties but not titled 'Coordinator'</t>
+        </is>
+      </c>
+      <c r="M103" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N103" s="8" t="inlineStr">
+        <is>
+          <t>Mentions full-cycle recruiting and proactive sourcing; lacks quantified daily call/screen metrics</t>
+        </is>
+      </c>
+      <c r="O103" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P103" s="8" t="inlineStr">
+        <is>
+          <t>Recruited for Analytics/Data Science, Account Managers, Marketing Ops; no SDRs, AEs, or BDRs</t>
+        </is>
+      </c>
+      <c r="Q103" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="R103" s="8" t="inlineStr">
+        <is>
+          <t>Accenture consulting with projects for Data &amp; AI, tech initiatives; SaaS-adjacent but not core product company</t>
+        </is>
+      </c>
+      <c r="S103" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="T103" s="8" t="inlineStr">
+        <is>
+          <t>B.E. Computer Engineering from GTU (2016); engineering background but no HR certifications</t>
+        </is>
+      </c>
+      <c r="U103" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="V103" s="8" t="inlineStr">
+        <is>
+          <t>Workforce Analytics and HR Consulting skills mentioned; no specific ATS tools (no Greenhouse) mentioned</t>
+        </is>
+      </c>
+      <c r="W103" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="X103" s="8" t="inlineStr">
+        <is>
+          <t>Mixed tenure: current 7 months, prior role 1.5 yrs, various 1-2 year stints; moderate stability</t>
+        </is>
+      </c>
+      <c r="Y103" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z103" s="8" t="inlineStr">
+        <is>
+          <t>Accenture US HQ but India-based role; some US stakeholder collaboration mentioned</t>
+        </is>
+      </c>
+      <c r="AA103" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB103" s="8" t="inlineStr">
+        <is>
+          <t>Career at large consulting/services firms (Accenture, dentsu, ALOIS); no VC-backed or startup experience</t>
+        </is>
+      </c>
+      <c r="AC103" s="8" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="AD103" s="8" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AE103" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF103" s="8" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="AG103" s="8" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="AH103" s="8" t="inlineStr">
+        <is>
+          <t>57.4%</t>
+        </is>
+      </c>
+      <c r="AI103" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AJ103" s="8" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+      <c r="AK103" s="8" t="inlineStr">
+        <is>
+          <t>• Ahmedabad-based with 8+ years recruiting experience
+• Full-cycle recruitment background with proactive sourcing
+• Engineering degree suggests technical awareness</t>
+        </is>
+      </c>
+      <c r="AL103" s="8" t="inlineStr">
+        <is>
+          <t>No Sales recruiting; limited pure SaaS exposure; no high-volume call metrics; no ATS/Greenhouse experience; consulting vs. product company background</t>
+        </is>
+      </c>
+      <c r="AM103" s="8" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="8" t="inlineStr">
+        <is>
+          <t>Anamika Pandit</t>
+        </is>
+      </c>
+      <c r="B104" s="8" t="inlineStr"/>
+      <c r="C104" s="8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/anamika-pandit-157883157</t>
+        </is>
+      </c>
+      <c r="D104" s="8" t="inlineStr">
+        <is>
+          <t>Senior Talent Acquisition Specialist</t>
+        </is>
+      </c>
+      <c r="E104" s="8" t="inlineStr">
+        <is>
+          <t>SUDERO ADVISORS AND CONSULTING</t>
+        </is>
+      </c>
+      <c r="F104" s="8" t="inlineStr">
+        <is>
+          <t>Bangalore, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="G104" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H104" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I104" s="8" t="inlineStr">
+        <is>
+          <t>BFSI/Banking industry majority (non-tech); No Gujarat/Gujarati connection; Zero SaaS/venture-backed tech exposure</t>
+        </is>
+      </c>
+      <c r="J104" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K104" s="8" t="inlineStr"/>
+      <c r="L104" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M104" s="8" t="inlineStr"/>
+      <c r="N104" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O104" s="8" t="inlineStr"/>
+      <c r="P104" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q104" s="8" t="inlineStr"/>
+      <c r="R104" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S104" s="8" t="inlineStr"/>
+      <c r="T104" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U104" s="8" t="inlineStr"/>
+      <c r="V104" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W104" s="8" t="inlineStr"/>
+      <c r="X104" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y104" s="8" t="inlineStr"/>
+      <c r="Z104" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA104" s="8" t="inlineStr"/>
+      <c r="AB104" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC104" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD104" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE104" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF104" s="8" t="inlineStr">
+        <is>
+          <t>52.8</t>
+        </is>
+      </c>
+      <c r="AG104" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AH104" s="8" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="AI104" s="8" t="inlineStr">
+        <is>
+          <t>Hard No</t>
+        </is>
+      </c>
+      <c r="AJ104" s="8" t="inlineStr"/>
+      <c r="AK104" s="8" t="inlineStr"/>
+      <c r="AL104" s="8" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="8" t="inlineStr">
+        <is>
+          <t>Iramben Saumil Virani</t>
+        </is>
+      </c>
+      <c r="B105" s="8" t="inlineStr"/>
+      <c r="C105" s="8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/iramben-saumil-virani-23110a21b</t>
+        </is>
+      </c>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Recruiter / US Recruiter</t>
+        </is>
+      </c>
+      <c r="E105" s="8" t="inlineStr">
+        <is>
+          <t>HGS / IMS People Possible</t>
+        </is>
+      </c>
+      <c r="F105" s="8" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat, India</t>
+        </is>
+      </c>
+      <c r="G105" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H105" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I105" s="8" t="inlineStr">
+        <is>
+          <t>Zero SaaS or Software Product exposure or worked at a venture backed technology company</t>
+        </is>
+      </c>
+      <c r="J105" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K105" s="8" t="inlineStr">
+        <is>
+          <t>Recruiter title, not Recruiting Coordinator; full-cycle but not coordination-focused</t>
+        </is>
+      </c>
+      <c r="L105" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M105" s="8" t="inlineStr">
+        <is>
+          <t>Quantified: 5-10 hires/quarter; high-volume projects (warehouse, logistics, healthcare, manufacturing); Fortune 100/500 clients</t>
+        </is>
+      </c>
+      <c r="N105" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O105" s="8" t="inlineStr">
+        <is>
+          <t>No evidence of Sales recruiting (SDRs, AEs, AMs, BDRs); recruited for IT, healthcare, warehouse, logistics</t>
+        </is>
+      </c>
+      <c r="P105" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q105" s="8" t="inlineStr">
+        <is>
+          <t>Zero SaaS exposure; career in staffing agency (IMS People Possible), BPO (HGS), and healthcare (Advantmed)</t>
+        </is>
+      </c>
+      <c r="R105" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S105" s="8" t="inlineStr">
+        <is>
+          <t>Master's degree in Food Science &amp; Nutrition from Gujarat University; not traditional HR education; no HR certifications mentioned</t>
+        </is>
+      </c>
+      <c r="T105" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U105" s="8" t="inlineStr">
+        <is>
+          <t>ATS experience: Bullhorn, Job Diva, E-recruit; coordination duties: onboarding, scheduling, candidate communication</t>
+        </is>
+      </c>
+      <c r="V105" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W105" s="8" t="inlineStr">
+        <is>
+          <t>HGS 6mo, IMS People Possible 11mo, Advantmed 11mo; pattern of short tenures and job-hopping</t>
+        </is>
+      </c>
+      <c r="X105" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y105" s="8" t="inlineStr">
+        <is>
+          <t>IMS People Possible: India company but US Recruiter role, worked with US-based Fortune 100/500 clients</t>
+        </is>
+      </c>
+      <c r="Z105" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA105" s="8" t="inlineStr">
+        <is>
+          <t>No VC-backed or startup experience; all companies established (BPO, staffing agency, healthcare)</t>
+        </is>
+      </c>
+      <c r="AB105" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AC105" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AD105" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AE105" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AF105" s="8" t="inlineStr">
+        <is>
+          <t>52.8</t>
+        </is>
+      </c>
+      <c r="AG105" s="8" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="AH105" s="8" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="AI105" s="8" t="inlineStr">
+        <is>
+          <t>Hard No</t>
+        </is>
+      </c>
+      <c r="AJ105" s="8" t="inlineStr"/>
+      <c r="AK105" s="8" t="inlineStr">
+        <is>
+          <t>No SaaS/tech background - auto-disqualified per JD requirements</t>
+        </is>
+      </c>
+      <c r="AL105" s="8" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="8" t="inlineStr">
+        <is>
+          <t>Yash Raj</t>
+        </is>
+      </c>
+      <c r="B106" s="8" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/yashrajsolanki</t>
+        </is>
+      </c>
+      <c r="D106" s="8" t="inlineStr">
+        <is>
+          <t>MSP Delivery Manager (North America)</t>
+        </is>
+      </c>
+      <c r="E106" s="8" t="inlineStr">
+        <is>
+          <t>Hirextra</t>
+        </is>
+      </c>
+      <c r="F106" s="8" t="inlineStr">
+        <is>
+          <t>Vadodara, Gujarat, India</t>
+        </is>
+      </c>
+      <c r="G106" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H106" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I106" s="8" t="inlineStr">
+        <is>
+          <t>Zero SaaS/Software/Venture-backed tech exposure — entire career in staffing agencies and MSP recruiting</t>
+        </is>
+      </c>
+      <c r="J106" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K106" s="8" t="inlineStr"/>
+      <c r="L106" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M106" s="8" t="inlineStr"/>
+      <c r="N106" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O106" s="8" t="inlineStr"/>
+      <c r="P106" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q106" s="8" t="inlineStr"/>
+      <c r="R106" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S106" s="8" t="inlineStr"/>
+      <c r="T106" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U106" s="8" t="inlineStr"/>
+      <c r="V106" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W106" s="8" t="inlineStr"/>
+      <c r="X106" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y106" s="8" t="inlineStr"/>
+      <c r="Z106" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA106" s="8" t="inlineStr"/>
+      <c r="AB106" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC106" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD106" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE106" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF106" s="8" t="inlineStr">
+        <is>
+          <t>52.8</t>
+        </is>
+      </c>
+      <c r="AG106" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AH106" s="8" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="AI106" s="8" t="inlineStr">
+        <is>
+          <t>Hard No</t>
+        </is>
+      </c>
+      <c r="AJ106" s="8" t="inlineStr"/>
+      <c r="AK106" s="8" t="inlineStr">
+        <is>
+          <t>No tech/SaaS exposure</t>
+        </is>
+      </c>
+      <c r="AL106" s="8" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="8" t="inlineStr">
+        <is>
+          <t>UNABLE_TO_EVALUATE</t>
+        </is>
+      </c>
+      <c r="B107" s="8" t="inlineStr"/>
+      <c r="C107" s="8" t="inlineStr"/>
+      <c r="D107" s="8" t="inlineStr"/>
+      <c r="E107" s="8" t="inlineStr"/>
+      <c r="F107" s="8" t="inlineStr"/>
+      <c r="G107" s="8" t="inlineStr"/>
+      <c r="H107" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I107" s="8" t="inlineStr">
+        <is>
+          <t>LinkedIn Recruiter access denied - profile ID AEMAAC56J-wBJLXiiRndjJJwPZq4Ekc0CwoPY4MM not accessible</t>
+        </is>
+      </c>
+      <c r="J107" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K107" s="8" t="inlineStr"/>
+      <c r="L107" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M107" s="8" t="inlineStr"/>
+      <c r="N107" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O107" s="8" t="inlineStr"/>
+      <c r="P107" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q107" s="8" t="inlineStr"/>
+      <c r="R107" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S107" s="8" t="inlineStr"/>
+      <c r="T107" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U107" s="8" t="inlineStr"/>
+      <c r="V107" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W107" s="8" t="inlineStr"/>
+      <c r="X107" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y107" s="8" t="inlineStr"/>
+      <c r="Z107" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA107" s="8" t="inlineStr"/>
+      <c r="AB107" s="8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AC107" s="8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AD107" s="8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE107" s="8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF107" s="8" t="inlineStr">
+        <is>
+          <t>52.8</t>
+        </is>
+      </c>
+      <c r="AG107" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AH107" s="8" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="AI107" s="8" t="inlineStr">
+        <is>
+          <t>Unable to Evaluate</t>
+        </is>
+      </c>
+      <c r="AJ107" s="8" t="inlineStr"/>
+      <c r="AK107" s="8" t="inlineStr"/>
+      <c r="AL107" s="8" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="8" t="inlineStr">
+        <is>
+          <t>Dhwani Saija</t>
+        </is>
+      </c>
+      <c r="B108" s="8" t="inlineStr"/>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/dhwani-saija-349466188</t>
+        </is>
+      </c>
+      <c r="D108" s="8" t="inlineStr">
+        <is>
+          <t>Sr Talent Acquisition &amp; Partner</t>
+        </is>
+      </c>
+      <c r="E108" s="8" t="inlineStr">
+        <is>
+          <t>E2M Solutions</t>
+        </is>
+      </c>
+      <c r="F108" s="8" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat, India</t>
+        </is>
+      </c>
+      <c r="G108" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H108" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I108" s="8" t="inlineStr">
+        <is>
+          <t>Zero SaaS/Software Product exposure — E2M Solutions is HR Services/recruiting firm, not tech SaaS company</t>
+        </is>
+      </c>
+      <c r="J108" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K108" s="8" t="inlineStr"/>
+      <c r="L108" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M108" s="8" t="inlineStr"/>
+      <c r="N108" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O108" s="8" t="inlineStr"/>
+      <c r="P108" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q108" s="8" t="inlineStr"/>
+      <c r="R108" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S108" s="8" t="inlineStr"/>
+      <c r="T108" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U108" s="8" t="inlineStr"/>
+      <c r="V108" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W108" s="8" t="inlineStr"/>
+      <c r="X108" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y108" s="8" t="inlineStr"/>
+      <c r="Z108" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA108" s="8" t="inlineStr"/>
+      <c r="AB108" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC108" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD108" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE108" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF108" s="8" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="AG108" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AH108" s="8" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="AI108" s="8" t="inlineStr">
+        <is>
+          <t>Hard No</t>
+        </is>
+      </c>
+      <c r="AJ108" s="8" t="inlineStr"/>
+      <c r="AK108" s="8" t="inlineStr">
+        <is>
+          <t>E2M Solutions is HR Services/recruiting, not tech SaaS</t>
+        </is>
+      </c>
+      <c r="AL108" s="8" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="8" t="inlineStr">
+        <is>
+          <t>Roger Sequeira</t>
+        </is>
+      </c>
+      <c r="B109" s="8" t="inlineStr"/>
+      <c r="C109" s="8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/roger-sequeira-01583424</t>
+        </is>
+      </c>
+      <c r="D109" s="8" t="inlineStr">
+        <is>
+          <t>Sr. Talent Acquisition</t>
+        </is>
+      </c>
+      <c r="E109" s="8" t="inlineStr">
+        <is>
+          <t>Microlink Solutions Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="F109" s="8" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat, India</t>
+        </is>
+      </c>
+      <c r="G109" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H109" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I109" s="8" t="inlineStr">
+        <is>
+          <t>Zero SaaS or Software Product exposure - all roles at IT Services companies</t>
+        </is>
+      </c>
+      <c r="J109" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K109" s="8" t="inlineStr">
+        <is>
+          <t>Sr. TA at IT services - not recruiting coordinator role</t>
+        </is>
+      </c>
+      <c r="L109" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M109" s="8" t="inlineStr"/>
+      <c r="N109" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O109" s="8" t="inlineStr"/>
+      <c r="P109" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q109" s="8" t="inlineStr"/>
+      <c r="R109" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S109" s="8" t="inlineStr"/>
+      <c r="T109" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U109" s="8" t="inlineStr"/>
+      <c r="V109" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W109" s="8" t="inlineStr"/>
+      <c r="X109" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y109" s="8" t="inlineStr"/>
+      <c r="Z109" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA109" s="8" t="inlineStr"/>
+      <c r="AB109" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AC109" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AD109" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AE109" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AF109" s="8" t="inlineStr">
+        <is>
+          <t>52.8</t>
+        </is>
+      </c>
+      <c r="AG109" s="8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AH109" s="8" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="AI109" s="8" t="inlineStr">
+        <is>
+          <t>Hard No</t>
+        </is>
+      </c>
+      <c r="AJ109" s="8" t="inlineStr"/>
+      <c r="AK109" s="8" t="inlineStr">
+        <is>
+          <t>Auto-disqualified: zero SaaS exposure</t>
+        </is>
+      </c>
+      <c r="AL109" s="8" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:AN1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
WebFetch Set as priority. Before splitting of agents
</commit_message>
<xml_diff>
--- a/_OUTPUT--Recruiting_Coord.xlsx
+++ b/_OUTPUT--Recruiting_Coord.xlsx
@@ -1035,7 +1035,7 @@
         <v>4</v>
       </c>
       <c r="AG3" s="8" t="n">
-        <v>43.4</v>
+        <v>43.40000000000001</v>
       </c>
       <c r="AH3" s="8" t="n">
         <v>53.4</v>
@@ -2039,7 +2039,7 @@
         <v>6</v>
       </c>
       <c r="AG9" s="5" t="n">
-        <v>39.1</v>
+        <v>39.09999999999999</v>
       </c>
       <c r="AH9" s="5" t="n">
         <v>53.4</v>
@@ -8659,7 +8659,7 @@
         </is>
       </c>
       <c r="AD51" s="8" t="n">
-        <v>39.8</v>
+        <v>0</v>
       </c>
       <c r="AE51" s="8" t="n">
         <v>2.4</v>
@@ -8668,24 +8668,24 @@
         <v>0</v>
       </c>
       <c r="AG51" s="8" t="n">
-        <v>42.2</v>
+        <v>2.4</v>
       </c>
       <c r="AH51" s="8" t="n">
-        <v>53.4</v>
+        <v>52.8</v>
       </c>
       <c r="AI51" s="8" t="inlineStr">
         <is>
-          <t>79.0%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="AJ51" s="8" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AK51" s="8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL51" s="8" t="inlineStr">
@@ -10055,7 +10055,7 @@
         </is>
       </c>
       <c r="AD60" s="8" t="n">
-        <v>36.9</v>
+        <v>0</v>
       </c>
       <c r="AE60" s="8" t="n">
         <v>2.4</v>
@@ -10064,24 +10064,24 @@
         <v>2</v>
       </c>
       <c r="AG60" s="8" t="n">
-        <v>41.3</v>
+        <v>4.4</v>
       </c>
       <c r="AH60" s="8" t="n">
-        <v>53.4</v>
+        <v>52.8</v>
       </c>
       <c r="AI60" s="8" t="inlineStr">
         <is>
-          <t>77.3%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="AJ60" s="8" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AK60" s="8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL60" s="8" t="inlineStr">
@@ -11181,7 +11181,7 @@
         </is>
       </c>
       <c r="AD67" s="10" t="n">
-        <v>37.2</v>
+        <v>0</v>
       </c>
       <c r="AE67" s="10" t="n">
         <v>2.4</v>
@@ -11190,24 +11190,24 @@
         <v>0</v>
       </c>
       <c r="AG67" s="10" t="n">
-        <v>39.6</v>
+        <v>2.4</v>
       </c>
       <c r="AH67" s="10" t="n">
-        <v>53.4</v>
+        <v>52.8</v>
       </c>
       <c r="AI67" s="10" t="inlineStr">
         <is>
-          <t>74.2%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="AJ67" s="10" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AK67" s="10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL67" s="10" t="inlineStr">
@@ -17118,36 +17118,42 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AD107" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE107" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF107" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG107" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH107" s="10" t="n">
-        <v>53.4</v>
+      <c r="AD107" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE107" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF107" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG107" s="10" t="inlineStr">
+        <is>
+          <t>52.8</t>
+        </is>
+      </c>
+      <c r="AH107" s="10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
       </c>
       <c r="AI107" s="10" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AJ107" s="10" t="inlineStr">
         <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="AK107" s="10" t="inlineStr">
-        <is>
-          <t>Hard No</t>
-        </is>
-      </c>
+          <t>Unable to Evaluate</t>
+        </is>
+      </c>
+      <c r="AK107" s="10" t="n"/>
       <c r="AL107" s="10" t="n"/>
       <c r="AM107" s="10" t="n"/>
       <c r="AN107" s="10" t="inlineStr">
@@ -18245,7 +18251,7 @@
         </is>
       </c>
       <c r="AD114" s="8" t="n">
-        <v>26.2</v>
+        <v>0</v>
       </c>
       <c r="AE114" s="8" t="n">
         <v>0</v>
@@ -18254,24 +18260,24 @@
         <v>2</v>
       </c>
       <c r="AG114" s="8" t="n">
-        <v>28.2</v>
+        <v>2</v>
       </c>
       <c r="AH114" s="8" t="n">
-        <v>53.4</v>
+        <v>52.8</v>
       </c>
       <c r="AI114" s="8" t="inlineStr">
         <is>
-          <t>52.8%</t>
+          <t>3.8%</t>
         </is>
       </c>
       <c r="AJ114" s="8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AK114" s="8" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL114" s="8" t="inlineStr">
@@ -18791,7 +18797,7 @@
         </is>
       </c>
       <c r="AD117" s="10" t="n">
-        <v>23.9</v>
+        <v>0</v>
       </c>
       <c r="AE117" s="10" t="n">
         <v>2.4</v>
@@ -18800,24 +18806,24 @@
         <v>0</v>
       </c>
       <c r="AG117" s="10" t="n">
-        <v>26.3</v>
+        <v>2.4</v>
       </c>
       <c r="AH117" s="10" t="n">
-        <v>53.4</v>
+        <v>52.8</v>
       </c>
       <c r="AI117" s="10" t="inlineStr">
         <is>
-          <t>49.3%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="AJ117" s="10" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AK117" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL117" s="10" t="inlineStr">
@@ -19123,7 +19129,7 @@
         </is>
       </c>
       <c r="AD119" s="10" t="n">
-        <v>23.3</v>
+        <v>0</v>
       </c>
       <c r="AE119" s="10" t="n">
         <v>2.4</v>
@@ -19132,24 +19138,24 @@
         <v>0</v>
       </c>
       <c r="AG119" s="10" t="n">
-        <v>25.7</v>
+        <v>2.4</v>
       </c>
       <c r="AH119" s="10" t="n">
-        <v>53.4</v>
+        <v>52.8</v>
       </c>
       <c r="AI119" s="10" t="inlineStr">
         <is>
-          <t>48.1%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="AJ119" s="10" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AK119" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL119" s="10" t="inlineStr">
@@ -20790,7 +20796,7 @@
         </is>
       </c>
       <c r="AD129" s="10" t="n">
-        <v>37.9</v>
+        <v>37.90000000000001</v>
       </c>
       <c r="AE129" s="10" t="n">
         <v>0.8</v>
@@ -33173,24 +33179,34 @@
           <t>Angel and Genie/datavuul appear startup-adjacent</t>
         </is>
       </c>
-      <c r="AD204" s="15" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="AE204" s="15" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AF204" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="AG204" s="15" t="n">
-        <v>21.4</v>
-      </c>
-      <c r="AH204" s="15" t="n">
-        <v>53.4</v>
+      <c r="AD204" s="15" t="inlineStr">
+        <is>
+          <t>17.2</t>
+        </is>
+      </c>
+      <c r="AE204" s="15" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="AF204" s="15" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="AG204" s="15" t="inlineStr">
+        <is>
+          <t>22.0</t>
+        </is>
+      </c>
+      <c r="AH204" s="15" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
       </c>
       <c r="AI204" s="15" t="inlineStr">
         <is>
-          <t>40.1%</t>
+          <t>41.2%</t>
         </is>
       </c>
       <c r="AJ204" s="15" t="inlineStr">
@@ -34011,24 +34027,34 @@
           <t>Primarily large platforms/agencies; minimal clear startup/VC exposure</t>
         </is>
       </c>
-      <c r="AD209" s="15" t="n">
-        <v>23.3</v>
-      </c>
-      <c r="AE209" s="15" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="AF209" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG209" s="15" t="n">
-        <v>27.7</v>
-      </c>
-      <c r="AH209" s="15" t="n">
-        <v>53.4</v>
+      <c r="AD209" s="15" t="inlineStr">
+        <is>
+          <t>23.3</t>
+        </is>
+      </c>
+      <c r="AE209" s="15" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="AF209" s="15" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="AG209" s="15" t="inlineStr">
+        <is>
+          <t>27.7</t>
+        </is>
+      </c>
+      <c r="AH209" s="15" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
       </c>
       <c r="AI209" s="15" t="inlineStr">
         <is>
-          <t>51.9%</t>
+          <t>51.88%</t>
         </is>
       </c>
       <c r="AJ209" s="15" t="inlineStr">
@@ -35598,7 +35624,7 @@
       </c>
       <c r="AN219" s="15" t="inlineStr">
         <is>
-          <t>DUPLICATE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -38721,7 +38747,7 @@
       </c>
       <c r="AI239" s="15" t="inlineStr">
         <is>
-          <t>70.0%</t>
+          <t>70%</t>
         </is>
       </c>
       <c r="AJ239" s="15" t="inlineStr">
@@ -41192,7 +41218,7 @@
       </c>
       <c r="AI255" s="15" t="inlineStr">
         <is>
-          <t>39.0%</t>
+          <t>39%</t>
         </is>
       </c>
       <c r="AJ255" s="15" t="inlineStr">
@@ -43030,7 +43056,7 @@
       </c>
       <c r="AI268" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ268" s="15" t="inlineStr">
@@ -43040,7 +43066,7 @@
       </c>
       <c r="AK268" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — Auto-DQ</t>
         </is>
       </c>
       <c r="AL268" s="15" t="inlineStr"/>
@@ -43156,7 +43182,7 @@
       </c>
       <c r="AI269" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ269" s="15" t="inlineStr">
@@ -43166,7 +43192,7 @@
       </c>
       <c r="AK269" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — Auto-DQ</t>
         </is>
       </c>
       <c r="AL269" s="15" t="inlineStr"/>
@@ -43282,7 +43308,7 @@
       </c>
       <c r="AI270" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ270" s="15" t="inlineStr">
@@ -43292,7 +43318,7 @@
       </c>
       <c r="AK270" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — Auto-DQ</t>
         </is>
       </c>
       <c r="AL270" s="15" t="inlineStr"/>
@@ -43408,7 +43434,7 @@
       </c>
       <c r="AI271" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ271" s="15" t="inlineStr">
@@ -43418,7 +43444,7 @@
       </c>
       <c r="AK271" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — Auto-DQ</t>
         </is>
       </c>
       <c r="AL271" s="15" t="inlineStr"/>
@@ -43566,17 +43592,17 @@
       </c>
       <c r="AI272" s="15" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="AJ272" s="15" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="AK272" s="15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Maybe</t>
         </is>
       </c>
       <c r="AL272" s="15" t="inlineStr">
@@ -43700,7 +43726,7 @@
       </c>
       <c r="AI273" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ273" s="15" t="inlineStr">
@@ -43710,7 +43736,7 @@
       </c>
       <c r="AK273" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — Auto-DQ</t>
         </is>
       </c>
       <c r="AL273" s="15" t="inlineStr"/>
@@ -43826,7 +43852,7 @@
       </c>
       <c r="AI274" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ274" s="15" t="inlineStr">
@@ -43836,7 +43862,7 @@
       </c>
       <c r="AK274" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — non-tech traditional industry recruiting (pharma mfg, coal &amp; mining, finance)</t>
         </is>
       </c>
       <c r="AL274" s="15" t="inlineStr"/>
@@ -43994,7 +44020,7 @@
       </c>
       <c r="AK275" s="15" t="inlineStr">
         <is>
-          <t>Strong Yes</t>
+          <t>Strong Yes — exact RC title at Lendingkart fintech (2yr), 3500-candidate high-volume hiring, Darwinbox + Greenhouse ATS, sales hiring experience</t>
         </is>
       </c>
       <c r="AL275" s="15" t="inlineStr">
@@ -44118,7 +44144,7 @@
       </c>
       <c r="AI276" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ276" s="15" t="inlineStr">
@@ -44128,7 +44154,7 @@
       </c>
       <c r="AK276" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — pure agency staffing (REQ Solutions) with healthcare sourcing, no in-house experience</t>
         </is>
       </c>
       <c r="AL276" s="15" t="inlineStr"/>
@@ -44244,7 +44270,7 @@
       </c>
       <c r="AI277" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ277" s="15" t="inlineStr">
@@ -44254,7 +44280,7 @@
       </c>
       <c r="AK277" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — pure agency staffing chain (Veterans Sourcing Group + IMS People Possible)</t>
         </is>
       </c>
       <c r="AL277" s="15" t="inlineStr"/>
@@ -44370,7 +44396,7 @@
       </c>
       <c r="AI278" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ278" s="15" t="inlineStr">
@@ -44380,7 +44406,7 @@
       </c>
       <c r="AK278" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — pure agency staffing (Placon HR Services), no in-house experience, still pursuing MBA</t>
         </is>
       </c>
       <c r="AL278" s="15" t="inlineStr"/>
@@ -44496,7 +44522,7 @@
       </c>
       <c r="AI279" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ279" s="15" t="inlineStr">
@@ -44506,7 +44532,7 @@
       </c>
       <c r="AK279" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — pure RPO agency (Horizon Talent Alliance), serving US staffing firms offshore</t>
         </is>
       </c>
       <c r="AL279" s="15" t="inlineStr"/>
@@ -44622,7 +44648,7 @@
       </c>
       <c r="AI280" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ280" s="15" t="inlineStr">
@@ -44632,7 +44658,7 @@
       </c>
       <c r="AK280" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — pure agency (iConsultera), healthcare staffing, accounting industry</t>
         </is>
       </c>
       <c r="AL280" s="15" t="inlineStr"/>
@@ -44748,7 +44774,7 @@
       </c>
       <c r="AI281" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ281" s="15" t="inlineStr">
@@ -44758,7 +44784,7 @@
       </c>
       <c r="AK281" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — pure agency chain (Confidential + LanceSoft), UK/Europe focus, contract/interim staffing</t>
         </is>
       </c>
       <c r="AL281" s="15" t="inlineStr"/>
@@ -44916,7 +44942,7 @@
       </c>
       <c r="AK282" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — very junior TA at legal services company, no high-volume/SaaS/sales hiring experience</t>
         </is>
       </c>
       <c r="AL282" s="15" t="inlineStr">
@@ -45040,7 +45066,7 @@
       </c>
       <c r="AI283" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ283" s="15" t="inlineStr">
@@ -45050,7 +45076,7 @@
       </c>
       <c r="AK283" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — pure agency chain (TalentCore + IMS Group), US IT staffing/bench sales</t>
         </is>
       </c>
       <c r="AL283" s="15" t="inlineStr"/>
@@ -45166,7 +45192,7 @@
       </c>
       <c r="AI284" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ284" s="15" t="inlineStr">
@@ -45176,7 +45202,7 @@
       </c>
       <c r="AK284" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — BPO background (Medusind AR Caller) + IMS People Possible agency chain</t>
         </is>
       </c>
       <c r="AL284" s="15" t="inlineStr"/>
@@ -45292,7 +45318,7 @@
       </c>
       <c r="AI285" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ285" s="15" t="inlineStr">
@@ -45302,7 +45328,7 @@
       </c>
       <c r="AK285" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — pure agency (Kyara Consulting), single role, no in-house experience</t>
         </is>
       </c>
       <c r="AL285" s="15" t="inlineStr"/>
@@ -45418,7 +45444,7 @@
       </c>
       <c r="AI286" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ286" s="15" t="inlineStr">
@@ -45428,7 +45454,7 @@
       </c>
       <c r="AK286" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — pure IMS People Possible agency (4yr+), UK staffing, no in-house experience</t>
         </is>
       </c>
       <c r="AL286" s="15" t="inlineStr"/>
@@ -45544,7 +45570,7 @@
       </c>
       <c r="AI287" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ287" s="15" t="inlineStr">
@@ -45554,7 +45580,7 @@
       </c>
       <c r="AK287" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — pure IMS Group agency (2yr 5mo), UK staffing operations</t>
         </is>
       </c>
       <c r="AL287" s="15" t="inlineStr"/>
@@ -45701,22 +45727,24 @@
       <c r="AG288" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="AH288" s="15" t="n">
-        <v>53.4</v>
+      <c r="AH288" s="15" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
       </c>
       <c r="AI288" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ288" s="15" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>DQ/F</t>
         </is>
       </c>
       <c r="AK288" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — primarily a teacher (6yr+), brief agency recruiter stint, education industry</t>
         </is>
       </c>
       <c r="AL288" s="15" t="inlineStr"/>
@@ -45863,22 +45891,24 @@
       <c r="AG289" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="AH289" s="15" t="n">
-        <v>53.4</v>
+      <c r="AH289" s="15" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
       </c>
       <c r="AI289" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ289" s="15" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>DQ/F</t>
         </is>
       </c>
       <c r="AK289" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — pure agency chain (IMS People Possible + Unity Systems), UK healthcare staffing</t>
         </is>
       </c>
       <c r="AL289" s="15" t="inlineStr"/>
@@ -46025,22 +46055,24 @@
       <c r="AG290" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="AH290" s="15" t="n">
-        <v>53.4</v>
+      <c r="AH290" s="15" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
       </c>
       <c r="AI290" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ290" s="15" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>DQ/F</t>
         </is>
       </c>
       <c r="AK290" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — pure IMS Group agency (4yr 6mo), pharma domain staffing</t>
         </is>
       </c>
       <c r="AL290" s="15" t="inlineStr"/>
@@ -46187,22 +46219,24 @@
       <c r="AG291" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="AH291" s="15" t="n">
-        <v>53.4</v>
+      <c r="AH291" s="15" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
       </c>
       <c r="AI291" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ291" s="15" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>DQ/F</t>
         </is>
       </c>
       <c r="AK291" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — pure IMS People Possible (2yr 9mo), healthcare/manufacturing/automotive staffing</t>
         </is>
       </c>
       <c r="AL291" s="15" t="inlineStr"/>
@@ -46360,7 +46394,7 @@
       </c>
       <c r="AK292" s="15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No — exact TA Coordinator title but only 4mo tenure, 17yr career gap, no relevant modern experience</t>
         </is>
       </c>
       <c r="AL292" s="15" t="inlineStr">
@@ -46515,22 +46549,24 @@
       <c r="AG293" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="AH293" s="15" t="n">
-        <v>53.4</v>
+      <c r="AH293" s="15" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
       </c>
       <c r="AI293" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ293" s="15" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>DQ/F</t>
         </is>
       </c>
       <c r="AK293" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — pure agency (Dangi Recruitment) + auto dealership sales background, very junior</t>
         </is>
       </c>
       <c r="AL293" s="15" t="inlineStr"/>
@@ -46843,22 +46879,24 @@
       <c r="AG295" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="AH295" s="15" t="n">
-        <v>53.4</v>
+      <c r="AH295" s="15" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
       </c>
       <c r="AI295" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ295" s="15" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>DQ/F</t>
         </is>
       </c>
       <c r="AK295" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — pure agency bench sales (Radiance Technologies), no recruiting background</t>
         </is>
       </c>
       <c r="AL295" s="15" t="inlineStr"/>
@@ -47010,17 +47048,17 @@
       </c>
       <c r="AI296" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ296" s="15" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>DQ/F</t>
         </is>
       </c>
       <c r="AK296" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — Auto-DQ</t>
         </is>
       </c>
       <c r="AL296" s="15" t="n"/>
@@ -47172,17 +47210,17 @@
       </c>
       <c r="AI297" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ297" s="15" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>DQ/F</t>
         </is>
       </c>
       <c r="AK297" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — Auto-DQ</t>
         </is>
       </c>
       <c r="AL297" s="15" t="n"/>
@@ -47334,17 +47372,17 @@
       </c>
       <c r="AI298" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ298" s="15" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>DQ/F</t>
         </is>
       </c>
       <c r="AK298" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — Auto-DQ</t>
         </is>
       </c>
       <c r="AL298" s="15" t="n"/>
@@ -47496,17 +47534,17 @@
       </c>
       <c r="AI299" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ299" s="15" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>DQ/F</t>
         </is>
       </c>
       <c r="AK299" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Hard No — Auto-DQ</t>
         </is>
       </c>
       <c r="AL299" s="15" t="n"/>
@@ -47827,34 +47865,44 @@
           <t>Auto-DQ</t>
         </is>
       </c>
-      <c r="AD301" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE301" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF301" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG301" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH301" t="n">
-        <v>53.4</v>
+      <c r="AD301" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE301" t="inlineStr">
+        <is>
+          <t>Auto-DQ</t>
+        </is>
+      </c>
+      <c r="AF301" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG301" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AH301" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="AI301" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AJ301" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>53.4</t>
         </is>
       </c>
       <c r="AK301" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AL301" t="inlineStr">
@@ -47943,26 +47991,12 @@
       <c r="AA302" s="15" t="inlineStr"/>
       <c r="AB302" s="15" t="inlineStr"/>
       <c r="AC302" s="15" t="inlineStr"/>
-      <c r="AD302" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE302" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF302" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG302" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH302" s="15" t="n">
-        <v>53.4</v>
-      </c>
-      <c r="AI302" s="15" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
+      <c r="AD302" s="15" t="inlineStr"/>
+      <c r="AE302" s="15" t="inlineStr"/>
+      <c r="AF302" s="15" t="inlineStr"/>
+      <c r="AG302" s="15" t="inlineStr"/>
+      <c r="AH302" s="15" t="inlineStr"/>
+      <c r="AI302" s="15" t="inlineStr"/>
       <c r="AJ302" s="15" t="inlineStr">
         <is>
           <t>F</t>
@@ -47975,11 +48009,7 @@
       </c>
       <c r="AL302" s="15" t="inlineStr"/>
       <c r="AM302" s="15" t="inlineStr"/>
-      <c r="AN302" s="15" t="inlineStr">
-        <is>
-          <t>DUPLICATE</t>
-        </is>
-      </c>
+      <c r="AN302" s="15" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" s="15" t="inlineStr">
@@ -48129,11 +48159,7 @@
       </c>
       <c r="AL303" s="15" t="inlineStr"/>
       <c r="AM303" s="15" t="inlineStr"/>
-      <c r="AN303" s="15" t="inlineStr">
-        <is>
-          <t>DUPLICATE</t>
-        </is>
-      </c>
+      <c r="AN303" s="15" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" s="15" t="inlineStr">
@@ -48255,36 +48281,24 @@
           <t>ZURU appears growth-stage tech but no explicit VC/YC mention; Ascension is large enterprise; minimal startup experience</t>
         </is>
       </c>
-      <c r="AD304" s="15" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="AE304" s="15" t="n">
-        <v>1.6</v>
+      <c r="AD304" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AE304" s="15" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
       </c>
       <c r="AF304" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG304" s="15" t="n">
-        <v>30.4</v>
-      </c>
-      <c r="AH304" s="15" t="n">
-        <v>53.4</v>
-      </c>
-      <c r="AI304" s="15" t="inlineStr">
-        <is>
-          <t>56.9%</t>
-        </is>
-      </c>
-      <c r="AJ304" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="AK304" s="15" t="inlineStr">
-        <is>
-          <t>Maybe</t>
-        </is>
-      </c>
+        <v>56.93</v>
+      </c>
+      <c r="AG304" s="15" t="inlineStr"/>
+      <c r="AH304" s="15" t="inlineStr"/>
+      <c r="AI304" s="15" t="inlineStr"/>
+      <c r="AJ304" s="15" t="inlineStr"/>
+      <c r="AK304" s="15" t="inlineStr"/>
       <c r="AL304" s="15" t="inlineStr"/>
       <c r="AM304" s="15" t="inlineStr"/>
       <c r="AN304" s="15" t="inlineStr"/>
@@ -48423,20 +48437,30 @@
           <t>Large enterprise/IT services background; no startup exposure evident</t>
         </is>
       </c>
-      <c r="AD305" s="15" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="AE305" s="15" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AF305" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG305" s="15" t="n">
-        <v>26.4</v>
-      </c>
-      <c r="AH305" s="15" t="n">
-        <v>53.4</v>
+      <c r="AD305" s="15" t="inlineStr">
+        <is>
+          <t>23.6</t>
+        </is>
+      </c>
+      <c r="AE305" s="15" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="AF305" s="15" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="AG305" s="15" t="inlineStr">
+        <is>
+          <t>26.4</t>
+        </is>
+      </c>
+      <c r="AH305" s="15" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
       </c>
       <c r="AI305" s="15" t="inlineStr">
         <is>
@@ -48589,20 +48613,30 @@
           <t>No clear startup/VC-backed company experience; self-employed consulting is not VC-backed</t>
         </is>
       </c>
-      <c r="AD306" s="15" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="AE306" s="15" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="AF306" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG306" s="15" t="n">
-        <v>26</v>
-      </c>
-      <c r="AH306" s="15" t="n">
-        <v>53.4</v>
+      <c r="AD306" s="15" t="inlineStr">
+        <is>
+          <t>21.6</t>
+        </is>
+      </c>
+      <c r="AE306" s="15" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="AF306" s="15" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="AG306" s="15" t="inlineStr">
+        <is>
+          <t>26.0</t>
+        </is>
+      </c>
+      <c r="AH306" s="15" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
       </c>
       <c r="AI306" s="15" t="inlineStr">
         <is>
@@ -48773,24 +48807,34 @@
           <t>No VC-backed or startup experience evident</t>
         </is>
       </c>
-      <c r="AD307" s="15" t="n">
-        <v>19.2</v>
-      </c>
-      <c r="AE307" s="15" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AF307" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG307" s="15" t="n">
-        <v>20</v>
-      </c>
-      <c r="AH307" s="15" t="n">
-        <v>53.4</v>
+      <c r="AD307" s="15" t="inlineStr">
+        <is>
+          <t>19.2</t>
+        </is>
+      </c>
+      <c r="AE307" s="15" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="AF307" s="15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG307" s="15" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="AH307" s="15" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
       </c>
       <c r="AI307" s="15" t="inlineStr">
         <is>
-          <t>37.5%</t>
+          <t>37.45%</t>
         </is>
       </c>
       <c r="AJ307" s="15" t="inlineStr">
@@ -49062,24 +49106,34 @@
           <t>Profile not accessible</t>
         </is>
       </c>
-      <c r="AD309" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE309" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF309" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG309" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH309" s="15" t="n">
-        <v>53.4</v>
+      <c r="AD309" s="15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE309" s="15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF309" s="15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG309" s="15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AH309" s="15" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
       </c>
       <c r="AI309" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ309" s="15" t="inlineStr">
@@ -49089,7 +49143,7 @@
       </c>
       <c r="AK309" s="15" t="inlineStr">
         <is>
-          <t>Hard No</t>
+          <t>Unable to Evaluate</t>
         </is>
       </c>
       <c r="AL309" s="15" t="inlineStr"/>
@@ -49286,11 +49340,6 @@
           <t>Career entirely in staffing agencies and IT services/non-product companies. No in-house recruiting coordinator experience at a product company. Adecco Group is a major staffing agency.</t>
         </is>
       </c>
-      <c r="AN310" t="inlineStr">
-        <is>
-          <t>DUPLICATE</t>
-        </is>
-      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -49433,24 +49482,34 @@
           <t>Large enterprise (Vodafone subsidiary), no startup</t>
         </is>
       </c>
-      <c r="AD311" t="n">
-        <v>11.2</v>
-      </c>
-      <c r="AE311" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF311" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG311" t="n">
-        <v>11.2</v>
-      </c>
-      <c r="AH311" t="n">
-        <v>53.4</v>
+      <c r="AD311" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="AE311" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF311" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG311" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="AH311" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
       </c>
       <c r="AI311" t="inlineStr">
         <is>
-          <t>21.0%</t>
+          <t>20.97%</t>
         </is>
       </c>
       <c r="AJ311" t="inlineStr">
@@ -49625,20 +49684,30 @@
           <t>Adani is large enterprise; CAVITAK unclear but appears staffing firm</t>
         </is>
       </c>
-      <c r="AD312" s="15" t="n">
-        <v>19.9</v>
-      </c>
-      <c r="AE312" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF312" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG312" s="15" t="n">
-        <v>19.9</v>
-      </c>
-      <c r="AH312" s="15" t="n">
-        <v>53.4</v>
+      <c r="AD312" s="15" t="inlineStr">
+        <is>
+          <t>19.9</t>
+        </is>
+      </c>
+      <c r="AE312" s="15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF312" s="15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG312" s="15" t="inlineStr">
+        <is>
+          <t>19.9</t>
+        </is>
+      </c>
+      <c r="AH312" s="15" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
       </c>
       <c r="AI312" s="15" t="inlineStr">
         <is>
@@ -49671,11 +49740,7 @@
           <t>0% SaaS fit; non-tech traditional industry background (Adani); no Sales hiring exposure</t>
         </is>
       </c>
-      <c r="AN312" s="15" t="inlineStr">
-        <is>
-          <t>DUPLICATE</t>
-        </is>
-      </c>
+      <c r="AN312" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>